<commit_message>
feat: add credit management functionality
- Implemented credit transactions handling in the application, allowing customers to convert refunds into credits or apply credits to subscriptions.
- Added a new CreditPanel component to manage credit transactions, including adding and deleting credits.
- Enhanced the CancelSubscriptionForm to include an option for keeping refunds as credits.
- Updated the PaymentPanel to allow applying credits to payments and handling credit payment reversals.
- Introduced utility functions for calculating credit balances and managing credit transactions.
- Updated data models and types to accommodate credit transactions.
- Added new Excel handling for credit transactions in the backend.
</commit_message>
<xml_diff>
--- a/data/test/customers.xlsx
+++ b/data/test/customers.xlsx
@@ -397,26 +397,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G51"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
         <v>name</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>phone</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>address</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>zone</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>notes</v>
-      </c>
-      <c r="F1" t="str">
-        <v>id</v>
       </c>
       <c r="G1" t="str">
         <v>createdAt</v>
@@ -424,27 +424,1016 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Phong</v>
+        <v>0901000001</v>
       </c>
       <c r="B2" t="str">
-        <v>123498712</v>
+        <v>Nguyễn Minh An</v>
       </c>
       <c r="C2" t="str">
-        <v>354 Ly Thuong Kiet</v>
+        <v>0901000001</v>
       </c>
       <c r="D2" t="str">
-        <v>Q10</v>
-      </c>
-      <c r="F2" t="str">
-        <v>123498712</v>
+        <v>12 Nguyễn Huệ, Bến Nghé, Quận 1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Q1</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-05-10T01:34:03.129Z</v>
+        <v>2025-09-04T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>0901000002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Trần Thị Lan</v>
+      </c>
+      <c r="C3" t="str">
+        <v>0901000002</v>
+      </c>
+      <c r="D3" t="str">
+        <v>56 Lê Lợi, Phường Bến Thành, Quận 1</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-09-09T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>0901000003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Lê Văn Tuấn</v>
+      </c>
+      <c r="C4" t="str">
+        <v>0901000003</v>
+      </c>
+      <c r="D4" t="str">
+        <v>78 Đinh Tiên Hoàng, Phường Đa Kao, Quận 1</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2025-09-14T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>0901000004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Phạm Thị Mai</v>
+      </c>
+      <c r="C5" t="str">
+        <v>0901000004</v>
+      </c>
+      <c r="D5" t="str">
+        <v>34 Trần Hưng Đạo, Phường Nguyễn Cư Trinh, Quận 1</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2025-09-19T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>0901000005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Hoàng Đức Hùng</v>
+      </c>
+      <c r="C6" t="str">
+        <v>0901000005</v>
+      </c>
+      <c r="D6" t="str">
+        <v>101 Lý Tự Trọng, Phường Bến Nghé, Quận 1</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2025-09-24T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>0901000006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Vũ Thị Hoa</v>
+      </c>
+      <c r="C7" t="str">
+        <v>0901000006</v>
+      </c>
+      <c r="D7" t="str">
+        <v>22 Võ Thị Sáu, Phường 7, Quận 3</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Q3</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2025-09-29T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>0901000007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Đặng Văn Dũng</v>
+      </c>
+      <c r="C8" t="str">
+        <v>0901000007</v>
+      </c>
+      <c r="D8" t="str">
+        <v>88 Nam Kỳ Khởi Nghĩa, Phường 8, Quận 3</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Q3</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2025-10-04T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>0901000008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Bùi Thị Linh</v>
+      </c>
+      <c r="C9" t="str">
+        <v>0901000008</v>
+      </c>
+      <c r="D9" t="str">
+        <v>15 Nguyễn Đình Chiểu, Phường 1, Quận 3</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Q3</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2025-10-09T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>0901000009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Ngô Quốc Nam</v>
+      </c>
+      <c r="C10" t="str">
+        <v>0901000009</v>
+      </c>
+      <c r="D10" t="str">
+        <v>30 Tôn Đức Thắng, Bến Nghé, Quận 1</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2025-10-14T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>0901000010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Hồ Thị Thảo</v>
+      </c>
+      <c r="C11" t="str">
+        <v>0901000010</v>
+      </c>
+      <c r="D11" t="str">
+        <v>8 Hai Bà Trưng, Bến Nghé, Quận 1</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2025-10-19T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>0901000011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Dương Minh Khoa</v>
+      </c>
+      <c r="C12" t="str">
+        <v>0901000011</v>
+      </c>
+      <c r="D12" t="str">
+        <v>200 Lê Văn Sỹ, Phường 14, Quận 3</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Q3</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Không ăn hải sản</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2025-10-24T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>0901000012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Lý Thị Ngọc</v>
+      </c>
+      <c r="C13" t="str">
+        <v>0901000012</v>
+      </c>
+      <c r="D13" t="str">
+        <v>45 Phan Xích Long, Phường 3, Phú Nhuận</v>
+      </c>
+      <c r="E13" t="str">
+        <v>PN</v>
+      </c>
+      <c r="G13" t="str">
+        <v>2025-10-29T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>0901000013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Phan Văn Long</v>
+      </c>
+      <c r="C14" t="str">
+        <v>0901000013</v>
+      </c>
+      <c r="D14" t="str">
+        <v>9 Hoàng Văn Thụ, Phường 8, Phú Nhuận</v>
+      </c>
+      <c r="E14" t="str">
+        <v>PN</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2025-11-03T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>0901000014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Trịnh Thị Thu</v>
+      </c>
+      <c r="C15" t="str">
+        <v>0901000014</v>
+      </c>
+      <c r="D15" t="str">
+        <v>33 Nguyễn Trọng Tuyển, Phường 10, Phú Nhuận</v>
+      </c>
+      <c r="E15" t="str">
+        <v>PN</v>
+      </c>
+      <c r="G15" t="str">
+        <v>2025-11-08T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>0901000015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Đinh Quang Bảo</v>
+      </c>
+      <c r="C16" t="str">
+        <v>0901000015</v>
+      </c>
+      <c r="D16" t="str">
+        <v>120 Điện Biên Phủ, Phường 15, Bình Thạnh</v>
+      </c>
+      <c r="E16" t="str">
+        <v>BT</v>
+      </c>
+      <c r="G16" t="str">
+        <v>2025-11-13T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>0901000016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Võ Thị Trang</v>
+      </c>
+      <c r="C17" t="str">
+        <v>0901000016</v>
+      </c>
+      <c r="D17" t="str">
+        <v>55 Bạch Đằng, Phường 2, Bình Thạnh</v>
+      </c>
+      <c r="E17" t="str">
+        <v>BT</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Dị ứng đậu phộng</v>
+      </c>
+      <c r="G17" t="str">
+        <v>2025-11-18T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>0901000017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Nguyễn Văn Kiên</v>
+      </c>
+      <c r="C18" t="str">
+        <v>0901000017</v>
+      </c>
+      <c r="D18" t="str">
+        <v>72 Nguyễn Gia Trí, Phường 25, Bình Thạnh</v>
+      </c>
+      <c r="E18" t="str">
+        <v>BT</v>
+      </c>
+      <c r="G18" t="str">
+        <v>2025-11-23T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>0901000018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Trần Thị Hương</v>
+      </c>
+      <c r="C19" t="str">
+        <v>0901000018</v>
+      </c>
+      <c r="D19" t="str">
+        <v>14 Hoàng Diệu, Phường 10, Quận 4</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Q4</v>
+      </c>
+      <c r="G19" t="str">
+        <v>2025-11-28T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>0901000019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Lê Minh Quân</v>
+      </c>
+      <c r="C20" t="str">
+        <v>0901000019</v>
+      </c>
+      <c r="D20" t="str">
+        <v>39 Tôn Thất Thuyết, Phường 16, Quận 4</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Q4</v>
+      </c>
+      <c r="G20" t="str">
+        <v>2025-12-03T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>0901000020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Phạm Thị Nhung</v>
+      </c>
+      <c r="C21" t="str">
+        <v>0901000020</v>
+      </c>
+      <c r="D21" t="str">
+        <v>67 Trần Xuân Soạn, Phường Tân Kiểng, Quận 7</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Q7</v>
+      </c>
+      <c r="G21" t="str">
+        <v>2025-12-08T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>0901000021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Huỳnh Văn Phúc</v>
+      </c>
+      <c r="C22" t="str">
+        <v>0901000021</v>
+      </c>
+      <c r="D22" t="str">
+        <v>5 Lê Thánh Tôn, Phường Bến Nghé, Quận 1</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G22" t="str">
+        <v>2025-12-13T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>0901000022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Đỗ Thị Phương</v>
+      </c>
+      <c r="C23" t="str">
+        <v>0901000022</v>
+      </c>
+      <c r="D23" t="str">
+        <v>200 Nguyễn Thị Minh Khai, Phường 6, Quận 3</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Q3</v>
+      </c>
+      <c r="G23" t="str">
+        <v>2025-12-18T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>0901000023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Cao Đức Anh</v>
+      </c>
+      <c r="C24" t="str">
+        <v>0901000023</v>
+      </c>
+      <c r="D24" t="str">
+        <v>88 Cộng Hòa, Phường 4, Tân Bình</v>
+      </c>
+      <c r="E24" t="str">
+        <v>TB</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Ăn chay thứ 2 và thứ 6</v>
+      </c>
+      <c r="G24" t="str">
+        <v>2025-12-23T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>0901000024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Mai Thị Yến</v>
+      </c>
+      <c r="C25" t="str">
+        <v>0901000024</v>
+      </c>
+      <c r="D25" t="str">
+        <v>120 Trường Chinh, Phường 12, Tân Bình</v>
+      </c>
+      <c r="E25" t="str">
+        <v>TB</v>
+      </c>
+      <c r="G25" t="str">
+        <v>2025-12-28T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>0901000025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Vũ Quang Hải</v>
+      </c>
+      <c r="C26" t="str">
+        <v>0901000025</v>
+      </c>
+      <c r="D26" t="str">
+        <v>44 Lê Trọng Tấn, Phường Tây Thạnh, Tân Phú</v>
+      </c>
+      <c r="E26" t="str">
+        <v>TP</v>
+      </c>
+      <c r="G26" t="str">
+        <v>2026-01-02T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>0901000026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Nguyễn Thị Bích</v>
+      </c>
+      <c r="C27" t="str">
+        <v>0901000026</v>
+      </c>
+      <c r="D27" t="str">
+        <v>66 Gò Vấp, Phường 3, Gò Vấp</v>
+      </c>
+      <c r="E27" t="str">
+        <v>GV</v>
+      </c>
+      <c r="G27" t="str">
+        <v>2026-01-07T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>0901000027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Trần Văn Thắng</v>
+      </c>
+      <c r="C28" t="str">
+        <v>0901000027</v>
+      </c>
+      <c r="D28" t="str">
+        <v>18 Phan Văn Trị, Phường 5, Gò Vấp</v>
+      </c>
+      <c r="E28" t="str">
+        <v>GV</v>
+      </c>
+      <c r="G28" t="str">
+        <v>2026-01-12T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>0901000028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Lê Thị Kim Anh</v>
+      </c>
+      <c r="C29" t="str">
+        <v>0901000028</v>
+      </c>
+      <c r="D29" t="str">
+        <v>90 Nguyễn Văn Nghi, Phường 7, Gò Vấp</v>
+      </c>
+      <c r="E29" t="str">
+        <v>GV</v>
+      </c>
+      <c r="G29" t="str">
+        <v>2026-01-17T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>0901000029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Phạm Quốc Việt</v>
+      </c>
+      <c r="C30" t="str">
+        <v>0901000029</v>
+      </c>
+      <c r="D30" t="str">
+        <v>15 Nguyễn Thị Thập, Phường Tân Phú, Quận 7</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Q7</v>
+      </c>
+      <c r="G30" t="str">
+        <v>2026-01-22T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>0901000030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Hoàng Thị Cúc</v>
+      </c>
+      <c r="C31" t="str">
+        <v>0901000030</v>
+      </c>
+      <c r="D31" t="str">
+        <v>30 Huỳnh Tấn Phát, Phường Phú Thuận, Quận 7</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Q7</v>
+      </c>
+      <c r="G31" t="str">
+        <v>2026-01-27T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>0901000031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Đặng Minh Tú</v>
+      </c>
+      <c r="C32" t="str">
+        <v>0901000031</v>
+      </c>
+      <c r="D32" t="str">
+        <v>45 Lý Chiêu Hoàng, Phường 10, Quận 6</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Q6</v>
+      </c>
+      <c r="G32" t="str">
+        <v>2026-02-01T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>0901000032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Bùi Văn Hòa</v>
+      </c>
+      <c r="C33" t="str">
+        <v>0901000032</v>
+      </c>
+      <c r="D33" t="str">
+        <v>77 Hậu Giang, Phường 11, Quận 6</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Q6</v>
+      </c>
+      <c r="G33" t="str">
+        <v>2026-02-06T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>0901000033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Ngô Thị Diễm</v>
+      </c>
+      <c r="C34" t="str">
+        <v>0901000033</v>
+      </c>
+      <c r="D34" t="str">
+        <v>100 Tô Ký, Phường Trung Mỹ Tây, Quận 12</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Q12</v>
+      </c>
+      <c r="G34" t="str">
+        <v>2026-02-11T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>0901000034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Hồ Văn Sơn</v>
+      </c>
+      <c r="C35" t="str">
+        <v>0901000034</v>
+      </c>
+      <c r="D35" t="str">
+        <v>55 Hà Huy Giáp, Phường Thạnh Lộc, Quận 12</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Q12</v>
+      </c>
+      <c r="G35" t="str">
+        <v>2026-02-16T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>0901000035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Dương Thị Lệ</v>
+      </c>
+      <c r="C36" t="str">
+        <v>0901000035</v>
+      </c>
+      <c r="D36" t="str">
+        <v>23 Lê Văn Việt, Phường Hiệp Phú, Thủ Đức</v>
+      </c>
+      <c r="E36" t="str">
+        <v>TD</v>
+      </c>
+      <c r="G36" t="str">
+        <v>2026-02-21T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>0901000036</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Lý Quốc Trung</v>
+      </c>
+      <c r="C37" t="str">
+        <v>0901000036</v>
+      </c>
+      <c r="D37" t="str">
+        <v>88 Võ Văn Ngân, Phường Bình Thọ, Thủ Đức</v>
+      </c>
+      <c r="E37" t="str">
+        <v>TD</v>
+      </c>
+      <c r="G37" t="str">
+        <v>2026-02-26T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>0901000037</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Phan Thị Nga</v>
+      </c>
+      <c r="C38" t="str">
+        <v>0901000037</v>
+      </c>
+      <c r="D38" t="str">
+        <v>12 Lê Văn Lương, Phước Kiểng, Nhà Bè</v>
+      </c>
+      <c r="E38" t="str">
+        <v>NB</v>
+      </c>
+      <c r="G38" t="str">
+        <v>2026-03-03T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>0901000038</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Trịnh Văn Hiếu</v>
+      </c>
+      <c r="C39" t="str">
+        <v>0901000038</v>
+      </c>
+      <c r="D39" t="str">
+        <v>34 Nguyễn Hữu Thọ, Phường Tân Hưng, Quận 7</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Q7</v>
+      </c>
+      <c r="G39" t="str">
+        <v>2026-03-08T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>0901000039</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Đinh Thị Xuân</v>
+      </c>
+      <c r="C40" t="str">
+        <v>0901000039</v>
+      </c>
+      <c r="D40" t="str">
+        <v>90 An Dương Vương, Phường An Lạc, Bình Tân</v>
+      </c>
+      <c r="E40" t="str">
+        <v>BTan</v>
+      </c>
+      <c r="G40" t="str">
+        <v>2026-03-13T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>0901000040</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Võ Minh Đạt</v>
+      </c>
+      <c r="C41" t="str">
+        <v>0901000040</v>
+      </c>
+      <c r="D41" t="str">
+        <v>120 Kinh Dương Vương, Phường 12, Bình Tân</v>
+      </c>
+      <c r="E41" t="str">
+        <v>BTan</v>
+      </c>
+      <c r="G41" t="str">
+        <v>2026-03-18T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>0901000041</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Nguyễn Thị Hằng</v>
+      </c>
+      <c r="C42" t="str">
+        <v>0901000041</v>
+      </c>
+      <c r="D42" t="str">
+        <v>12 Nguyễn Huệ, Bến Nghé, Quận 1</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G42" t="str">
+        <v>2026-03-23T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>0901000042</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Trần Quang Trung</v>
+      </c>
+      <c r="C43" t="str">
+        <v>0901000042</v>
+      </c>
+      <c r="D43" t="str">
+        <v>56 Lê Lợi, Phường Bến Thành, Quận 1</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G43" t="str">
+        <v>2026-03-28T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>0901000043</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Lê Thị Mỹ Duyên</v>
+      </c>
+      <c r="C44" t="str">
+        <v>0901000043</v>
+      </c>
+      <c r="D44" t="str">
+        <v>78 Đinh Tiên Hoàng, Phường Đa Kao, Quận 1</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G44" t="str">
+        <v>2026-04-02T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>0901000044</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Phạm Văn Tài</v>
+      </c>
+      <c r="C45" t="str">
+        <v>0901000044</v>
+      </c>
+      <c r="D45" t="str">
+        <v>34 Trần Hưng Đạo, Phường Nguyễn Cư Trinh, Quận 1</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G45" t="str">
+        <v>2026-04-07T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>0901000045</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Huỳnh Thị Loan</v>
+      </c>
+      <c r="C46" t="str">
+        <v>0901000045</v>
+      </c>
+      <c r="D46" t="str">
+        <v>101 Lý Tự Trọng, Phường Bến Nghé, Quận 1</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G46" t="str">
+        <v>2026-04-12T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>0901000046</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Đỗ Văn Khải</v>
+      </c>
+      <c r="C47" t="str">
+        <v>0901000046</v>
+      </c>
+      <c r="D47" t="str">
+        <v>22 Võ Thị Sáu, Phường 7, Quận 3</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Q3</v>
+      </c>
+      <c r="G47" t="str">
+        <v>2026-04-17T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>0901000047</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Cao Thị Bảo Châu</v>
+      </c>
+      <c r="C48" t="str">
+        <v>0901000047</v>
+      </c>
+      <c r="D48" t="str">
+        <v>88 Nam Kỳ Khởi Nghĩa, Phường 8, Quận 3</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Q3</v>
+      </c>
+      <c r="G48" t="str">
+        <v>2026-04-22T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>0901000048</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Mai Văn Lợi</v>
+      </c>
+      <c r="C49" t="str">
+        <v>0901000048</v>
+      </c>
+      <c r="D49" t="str">
+        <v>15 Nguyễn Đình Chiểu, Phường 1, Quận 3</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Q3</v>
+      </c>
+      <c r="G49" t="str">
+        <v>2026-04-27T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>0901000049</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Vũ Thị Thanh Hà</v>
+      </c>
+      <c r="C50" t="str">
+        <v>0901000049</v>
+      </c>
+      <c r="D50" t="str">
+        <v>30 Tôn Đức Thắng, Bến Nghé, Quận 1</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G50" t="str">
+        <v>2026-05-02T08:41:15.938Z</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>0901000050</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Nguyễn Đức Toàn</v>
+      </c>
+      <c r="C51" t="str">
+        <v>0901000050</v>
+      </c>
+      <c r="D51" t="str">
+        <v>8 Hai Bà Trưng, Bến Nghé, Quận 1</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Q1</v>
+      </c>
+      <c r="G51" t="str">
+        <v>2026-05-07T08:41:15.938Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G51"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>